<commit_message>
main6: PDF Yok-In dkk. 2026 diperoleh; label C1-nya dari teks lengkap
- PDF yokin20263d (diunduh peninjau lewat peramban) serta Cherie 2015 (dua)
  dan Junior 2023 ditambahkan beserta teksnya. PDF teks lengkap 480 dari
  1.013; kajian C1 dengan teks lengkap 198 dari 199, tinggal Safre dkk. 2024.
- Label Yok-In dikukuhkan dari teks lengkap (M4, S, tidak per kelas; Tabel 4
  dan 6), disetujui peninjau 20 Oktober 2026. Lampiran A kini "Full text".
- Kalimat naskah tentang kajian tanpa teks lengkap diubah ke bentuk tunggal.
- verifikasi_log_manusia.py: nilai halaman "Abstrak (...null...)" tidak lagi
  diterjemahkan menjadi "hanya judul".
</commit_message>
<xml_diff>
--- a/literature/scopus-2026-09/verifikasi/cek-4-teks-lengkap/PERMINTAAN-PDF-BU-FATMA.xlsx
+++ b/literature/scopus-2026-09/verifikasi/cek-4-teks-lengkap/PERMINTAAN-PDF-BU-FATMA.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Permintaan PDF" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Permintaan PDF'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Permintaan PDF'!$A$1:$L$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -581,222 +581,10 @@
       </c>
       <c r="L2" s="2" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>C1 lainnya</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Yok-In K.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>3D reconstruction and segmentation of grape bunches for robotic berry thinning</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Computers and Electronics in Agriculture</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Elsevier</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>10.1016/j.compag.2026.111898</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>yokin20263d.pdf</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>C3 multipandang</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Junior F.A.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Video based oil palm ripeness detection model using deep learning</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Heliyon</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Elsevier</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>10.1016/j.heliyon.2023.e13036</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>junior2023video.pdf</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>C3 multipandang</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>2015</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Cherie D.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Advance models for camera-vision based oil content prediction of intact oil palm fruits (Elaeis Guineensis Jacq) on trees with nondestructive evaluation</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>International Journal on Advanced Science Engineering and Information Technology</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>International Journal on Advanced Science Engineering and Information Technology</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>10.18517/ijaseit.5.4.542</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>cherie2015advance.pdf</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>C3 multipandang</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>2015</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Cherie D.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Optical characteristics of oil palm fresh fruits bunch (FFB) under three spectrum regions influence for harvest decision</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>International Journal on Advanced Science Engineering and Information Technology</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>International Journal on Advanced Science Engineering and Information Technology</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>10.18517/ijaseit.5.3.534</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>cherie2015optical.pdf</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L2"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>